<commit_message>
fix: some of the datasets had incorrect entries
</commit_message>
<xml_diff>
--- a/src/cubes/data/materials/Materials_extended.xlsx
+++ b/src/cubes/data/materials/Materials_extended.xlsx
@@ -5,20 +5,20 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannes/Work/elizabeth-homes/src/cubes/data/materials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/JackLynch/Documents/CUBES/src/cubes/data/materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFE7E4AA-5081-6A46-9729-69BC8BD5B20F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3A969D9-3675-0C46-9B87-455685FA5096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="13860" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$A$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$A$31</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
   <si>
     <t>Material</t>
   </si>
@@ -176,7 +176,13 @@
     <t>Cement fiber slabs shredded wood</t>
   </si>
   <si>
-    <t>Asbestos fiber</t>
+    <t>Brick fired clay 1280</t>
+  </si>
+  <si>
+    <t>Brick</t>
+  </si>
+  <si>
+    <t>Asbestos fibre</t>
   </si>
 </sst>
 </file>
@@ -558,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.1640625" customWidth="1"/>
@@ -628,7 +634,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B3" s="4">
         <v>0.06</v>
@@ -643,19 +649,19 @@
         <v>9</v>
       </c>
       <c r="F3" t="str">
-        <f t="shared" ref="F3:F30" si="0">F2</f>
+        <f t="shared" ref="F3:F31" si="0">F2</f>
         <v>Rough</v>
       </c>
       <c r="G3">
-        <f t="shared" ref="G3:G30" si="1">G2</f>
+        <f t="shared" ref="G3:G31" si="1">G2</f>
         <v>0.9</v>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H30" si="2">H2</f>
+        <f t="shared" ref="H3:H31" si="2">H2</f>
         <v>0.7</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I30" si="3">I2</f>
+        <f t="shared" ref="I3:I31" si="3">I2</f>
         <v>0.7</v>
       </c>
     </row>
@@ -1255,85 +1261,81 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="B22" s="4">
-        <v>0.41</v>
+        <v>0.48</v>
       </c>
       <c r="C22" s="5">
-        <v>1120</v>
+        <v>1280</v>
       </c>
       <c r="D22" s="5">
         <v>800</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F22" t="str">
-        <f t="shared" si="0"/>
-        <v>Rough</v>
+        <v>46</v>
+      </c>
+      <c r="F22" t="s">
+        <v>10</v>
       </c>
       <c r="G22">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="H22">
-        <f t="shared" si="2"/>
         <v>0.7</v>
       </c>
       <c r="I22">
-        <f t="shared" si="3"/>
         <v>0.7</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23" s="4">
-        <v>3.49</v>
+        <v>0.41</v>
       </c>
       <c r="C23" s="5">
-        <v>2880</v>
+        <v>1120</v>
       </c>
       <c r="D23" s="5">
-        <v>840</v>
+        <v>800</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F23" t="str">
-        <f t="shared" si="0"/>
+        <f>F21</f>
         <v>Rough</v>
       </c>
       <c r="G23">
-        <f t="shared" si="1"/>
+        <f>G21</f>
         <v>0.9</v>
       </c>
       <c r="H23">
-        <f t="shared" si="2"/>
+        <f>H21</f>
         <v>0.7</v>
       </c>
       <c r="I23">
-        <f t="shared" si="3"/>
+        <f>I21</f>
         <v>0.7</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B24" s="4">
-        <v>2.4900000000000002</v>
+        <v>3.49</v>
       </c>
       <c r="C24" s="5">
-        <v>2650</v>
+        <v>2880</v>
       </c>
       <c r="D24" s="5">
-        <v>900</v>
+        <v>840</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F24" t="str">
         <f t="shared" si="0"/>
@@ -1354,19 +1356,19 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B25" s="4">
-        <v>1.83</v>
+        <v>2.4900000000000002</v>
       </c>
       <c r="C25" s="5">
-        <v>2200</v>
+        <v>2650</v>
       </c>
       <c r="D25" s="5">
-        <v>710</v>
+        <v>900</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F25" t="str">
         <f t="shared" si="0"/>
@@ -1387,19 +1389,19 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B26" s="4">
-        <v>1.5</v>
+        <v>1.83</v>
       </c>
       <c r="C26" s="5">
-        <v>2180</v>
+        <v>2200</v>
       </c>
       <c r="D26" s="5">
-        <v>720</v>
+        <v>710</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F26" t="str">
         <f t="shared" si="0"/>
@@ -1420,16 +1422,16 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B27" s="4">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="C27" s="5">
-        <v>2000</v>
+        <v>2180</v>
       </c>
       <c r="D27" s="5">
-        <v>840</v>
+        <v>720</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>35</v>
@@ -1453,19 +1455,19 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B28" s="4">
-        <v>0.23</v>
+        <v>1.2</v>
       </c>
       <c r="C28" s="5">
-        <v>650</v>
+        <v>2000</v>
       </c>
       <c r="D28" s="5">
-        <v>3050</v>
+        <v>840</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F28" t="str">
         <f t="shared" si="0"/>
@@ -1486,19 +1488,19 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B29" s="4">
-        <v>0.16</v>
+        <v>0.23</v>
       </c>
       <c r="C29" s="5">
-        <v>720</v>
+        <v>650</v>
       </c>
       <c r="D29" s="5">
-        <v>1260</v>
+        <v>3050</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F29" t="str">
         <f t="shared" si="0"/>
@@ -1519,16 +1521,16 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B30" s="4">
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="C30" s="5">
         <v>720</v>
       </c>
       <c r="D30" s="5">
-        <v>1680</v>
+        <v>1260</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>42</v>
@@ -1546,6 +1548,39 @@
         <v>0.7</v>
       </c>
       <c r="I30">
+        <f t="shared" si="3"/>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="4">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="C31" s="5">
+        <v>720</v>
+      </c>
+      <c r="D31" s="5">
+        <v>1680</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F31" t="str">
+        <f t="shared" si="0"/>
+        <v>Rough</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="1"/>
+        <v>0.9</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="2"/>
+        <v>0.7</v>
+      </c>
+      <c r="I31">
         <f t="shared" si="3"/>
         <v>0.7</v>
       </c>

</xml_diff>